<commit_message>
Update Scen_Par-SYS_FF2price - OilCopy.xlsx
Oil price increase by 2
</commit_message>
<xml_diff>
--- a/SuppXLS/Scen_Par-SYS_FF2price - OilCopy.xlsx
+++ b/SuppXLS/Scen_Par-SYS_FF2price - OilCopy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BSuleimenov\Documents\GitHub\times-ireland-model\SuppXLS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git Folder\Project\times-ireland-model\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87FDBEF-FABF-4698-9580-5EEC6465C730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FBD53C8-9B0C-428B-8385-0DA7E6BA26D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="24" r:id="rId1"/>
@@ -138,7 +138,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="90">
   <si>
     <t>LimType</t>
   </si>
@@ -415,9 +415,6 @@
     <t>IRE_PRICE</t>
   </si>
   <si>
-    <t>IMPOIL*,IMPGAS*</t>
-  </si>
-  <si>
     <t>AllRegions</t>
   </si>
   <si>
@@ -427,7 +424,10 @@
     <t>ELC, BIO</t>
   </si>
   <si>
-    <t>IMPELC*,IMPBIO*</t>
+    <t>*2</t>
+  </si>
+  <si>
+    <t>IMPOIL*</t>
   </si>
 </sst>
 </file>
@@ -5041,7 +5041,7 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.3">
@@ -5057,7 +5057,7 @@
         <v>81</v>
       </c>
       <c r="J6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
@@ -5216,7 +5216,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2314F01-B0DB-448B-9217-DEB90E2D1CCA}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="B2:AM10"/>
+  <dimension ref="B2:AM5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
@@ -5241,7 +5241,7 @@
         <v>63</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>61</v>
@@ -5258,12 +5258,11 @@
       <c r="D4" t="s">
         <v>84</v>
       </c>
-      <c r="E4" t="str">
-        <f>"*"&amp;VLOOKUP(config!$B$3,config!$H$6:$I$12,2,FALSE)</f>
-        <v>*1.5</v>
+      <c r="E4" t="s">
+        <v>88</v>
       </c>
       <c r="G4" s="26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H4" s="26"/>
       <c r="I4" s="26"/>
@@ -5299,16 +5298,7 @@
       <c r="AM4" s="26"/>
     </row>
     <row r="5" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="D5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" t="str">
-        <f>"*"&amp;VLOOKUP(config!$B$3,config!$H$6:$J$12,3,FALSE)</f>
-        <v>*1.375</v>
-      </c>
-      <c r="G5" s="26" t="s">
-        <v>89</v>
-      </c>
+      <c r="G5" s="26"/>
       <c r="H5" s="26"/>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
@@ -5342,11 +5332,6 @@
       <c r="AL5" s="26"/>
       <c r="AM5" s="26"/>
     </row>
-    <row r="10" spans="2:39" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>1000</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>